<commit_message>
feat: update test automation and documentation for new features
Updated test cases for new Pro waitlist and CFP submission flows; adjusted test plan descriptions to reflect changes.

Co-authored-by: Salvador A. Sánchez Campos <58109205+SalvadorSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/evoca-test-plan.xlsx
+++ b/docs/evoca-test-plan.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="353">
   <si>
     <t>Evoca — Test Plan</t>
   </si>
@@ -531,30 +531,30 @@
     <t>/cfp/[slug]</t>
   </si>
   <si>
+    <t>features-public.spec.ts › CFP public submission (renders, validation, confirm)</t>
+  </si>
+  <si>
+    <t>TC-021</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>Rate + accept proposal</t>
+  </si>
+  <si>
+    <t>Open review board, rate, accept one</t>
+  </si>
+  <si>
+    <t>Creates unscheduled slot + pending affiliation</t>
+  </si>
+  <si>
+    <t>/dashboard/conference/[id]/cfp/review</t>
+  </si>
+  <si>
     <t>Manual</t>
   </si>
   <si>
-    <t>CFP public submission (manual QA)</t>
-  </si>
-  <si>
-    <t>TC-021</t>
-  </si>
-  <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>Rate + accept proposal</t>
-  </si>
-  <si>
-    <t>Open review board, rate, accept one</t>
-  </si>
-  <si>
-    <t>Creates unscheduled slot + pending affiliation</t>
-  </si>
-  <si>
-    <t>/dashboard/conference/[id]/cfp/review</t>
-  </si>
-  <si>
     <t>CFP review board (manual QA)</t>
   </si>
   <si>
@@ -696,7 +696,7 @@
     <t>/remote/[token]</t>
   </si>
   <si>
-    <t>features-live.spec.ts › Speaker phone remote</t>
+    <t>features-live.spec.ts › invalid token gate (valid load needs live session)</t>
   </si>
   <si>
     <t>TC-029</t>
@@ -735,7 +735,7 @@
     <t>/qna/[sessionId]</t>
   </si>
   <si>
-    <t>features-live.spec.ts › Q&amp;A attendee view</t>
+    <t>Q&amp;A submit (manual QA — needs live PartyKit client round-trip)</t>
   </si>
   <si>
     <t>TC-031</t>
@@ -792,7 +792,7 @@
     <t>/wall</t>
   </si>
   <si>
-    <t>features-live.spec.ts › Live wall</t>
+    <t>Live wall (manual QA — needs live PartyKit broadcast)</t>
   </si>
   <si>
     <t>TC-034</t>
@@ -1027,6 +1027,24 @@
   </si>
   <si>
     <t>features-public.spec.ts › Theme switcher (feat-011)</t>
+  </si>
+  <si>
+    <t>TC-046</t>
+  </si>
+  <si>
+    <t>Pro waitlist</t>
+  </si>
+  <si>
+    <t>Speaker Pro waitlist capture</t>
+  </si>
+  <si>
+    <t>On /pricing (Speakers), submit empty / valid / duplicate email</t>
+  </si>
+  <si>
+    <t>Inline error on empty; success state on valid; duplicate message on 409</t>
+  </si>
+  <si>
+    <t>features-public.spec.ts › Pro waitlist (empty/valid/duplicate states)</t>
   </si>
   <si>
     <t>Count</t>
@@ -1655,7 +1673,7 @@
   <sheetPr>
     <tabColor rgb="FF0A0A0A"/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -2640,11 +2658,11 @@
       <c r="I21" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="J21" s="9" t="s">
+      <c r="J21" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="K21" s="6" t="s">
         <v>172</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>173</v>
       </c>
       <c r="L21" s="6" t="s">
         <v>47</v>
@@ -2661,34 +2679,34 @@
     </row>
     <row r="22" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>159</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>177</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>178</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>52</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>44</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>180</v>
@@ -2714,7 +2732,7 @@
         <v>159</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>182</v>
@@ -2729,13 +2747,13 @@
         <v>52</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="I23" s="6" t="s">
         <v>54</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K23" s="6" t="s">
         <v>185</v>
@@ -2923,7 +2941,7 @@
         <v>54</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K27" s="6" t="s">
         <v>212</v>
@@ -2970,7 +2988,7 @@
         <v>44</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K28" s="3" t="s">
         <v>220</v>
@@ -3110,8 +3128,8 @@
       <c r="I31" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="J31" s="8" t="s">
-        <v>116</v>
+      <c r="J31" s="9" t="s">
+        <v>179</v>
       </c>
       <c r="K31" s="6" t="s">
         <v>240</v>
@@ -3205,7 +3223,7 @@
         <v>44</v>
       </c>
       <c r="J33" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K33" s="6" t="s">
         <v>252</v>
@@ -3251,8 +3269,8 @@
       <c r="I34" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="J34" s="8" t="s">
-        <v>116</v>
+      <c r="J34" s="9" t="s">
+        <v>179</v>
       </c>
       <c r="K34" s="3" t="s">
         <v>259</v>
@@ -3393,7 +3411,7 @@
         <v>44</v>
       </c>
       <c r="J37" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K37" s="6" t="s">
         <v>279</v>
@@ -3675,7 +3693,7 @@
         <v>54</v>
       </c>
       <c r="J43" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K43" s="6" t="s">
         <v>318</v>
@@ -3722,7 +3740,7 @@
         <v>54</v>
       </c>
       <c r="J44" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K44" s="3" t="s">
         <v>324</v>
@@ -3769,7 +3787,7 @@
         <v>330</v>
       </c>
       <c r="J45" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="K45" s="6" t="s">
         <v>331</v>
@@ -3834,9 +3852,56 @@
         <v>1</v>
       </c>
     </row>
+    <row r="47" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="L47" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="M47" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="N47" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="O47" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O1"/>
-  <conditionalFormatting sqref="L2:L46">
+  <conditionalFormatting sqref="L2:L47">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("Pass",L2)))</formula>
     </cfRule>
@@ -3848,10 +3913,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="L10:L46">
+    <dataValidation type="list" sqref="L10:L47">
       <formula1>"Not Started,Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="L2:L46">
+    <dataValidation type="list" sqref="L2:L47">
       <formula1>"Not Started,Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3878,10 +3943,10 @@
         <v>33</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3889,62 +3954,62 @@
         <v>47</v>
       </c>
       <c r="B2">
-        <f>COUNTIF('Test Plan'!L2:L46,"Not Started")</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"Not Started")</f>
       </c>
       <c r="C2" s="10">
-        <f>COUNTIF('Test Plan'!L2:L46,"Not Started")/45</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"Not Started")/46</f>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="B3">
-        <f>COUNTIF('Test Plan'!L2:L46,"Pass")</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"Pass")</f>
       </c>
       <c r="C3" s="10">
-        <f>COUNTIF('Test Plan'!L2:L46,"Pass")/45</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"Pass")/46</f>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="B4">
-        <f>COUNTIF('Test Plan'!L2:L46,"Fail")</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"Fail")</f>
       </c>
       <c r="C4" s="10">
-        <f>COUNTIF('Test Plan'!L2:L46,"Fail")/45</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"Fail")/46</f>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Plan'!L2:L46,"Blocked")</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"Blocked")</f>
       </c>
       <c r="C5" s="10">
-        <f>COUNTIF('Test Plan'!L2:L46,"Blocked")/45</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"Blocked")/46</f>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Plan'!L2:L46,"N/A")</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"N/A")</f>
       </c>
       <c r="C6" s="10">
-        <f>COUNTIF('Test Plan'!L2:L46,"N/A")/45</f>
+        <f>COUNTIF('Test Plan'!L2:L47,"N/A")/46</f>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B8" s="11">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
@@ -3952,13 +4017,13 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>345</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3966,10 +4031,10 @@
         <v>45</v>
       </c>
       <c r="B11">
-        <f>COUNTIF('Test Plan'!J2:J46,"E2E")</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"E2E")</f>
       </c>
       <c r="C11" s="10">
-        <f>COUNTIF('Test Plan'!J2:J46,"E2E")/45</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"E2E")/46</f>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -3977,10 +4042,10 @@
         <v>109</v>
       </c>
       <c r="B12">
-        <f>COUNTIF('Test Plan'!J2:J46,"Unit + E2E")</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"Unit + E2E")</f>
       </c>
       <c r="C12" s="10">
-        <f>COUNTIF('Test Plan'!J2:J46,"Unit + E2E")/45</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"Unit + E2E")/46</f>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3988,10 +4053,10 @@
         <v>116</v>
       </c>
       <c r="B13">
-        <f>COUNTIF('Test Plan'!J2:J46,"E2E (smoke)")</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"E2E (smoke)")</f>
       </c>
       <c r="C13" s="10">
-        <f>COUNTIF('Test Plan'!J2:J46,"E2E (smoke)")/45</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"E2E (smoke)")/46</f>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3999,32 +4064,32 @@
         <v>82</v>
       </c>
       <c r="B14">
-        <f>COUNTIF('Test Plan'!J2:J46,"Unit")</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"Unit")</f>
       </c>
       <c r="C14" s="10">
-        <f>COUNTIF('Test Plan'!J2:J46,"Unit")/45</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"Unit")/46</f>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B15">
-        <f>COUNTIF('Test Plan'!J2:J46,"Manual")</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"Manual")</f>
       </c>
       <c r="C15" s="10">
-        <f>COUNTIF('Test Plan'!J2:J46,"Manual")/45</f>
+        <f>COUNTIF('Test Plan'!J2:J47,"Manual")/46</f>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="B16" s="11">
-        <f>45-COUNTIF('Test Plan'!J2:J46,"Manual")</f>
+        <f>46-COUNTIF('Test Plan'!J2:J47,"Manual")</f>
       </c>
       <c r="C16" s="12">
-        <f>(45-COUNTIF('Test Plan'!J2:J46,"Manual"))/45</f>
+        <f>(46-COUNTIF('Test Plan'!J2:J47,"Manual"))/46</f>
       </c>
     </row>
   </sheetData>

</xml_diff>